<commit_message>
Generate Q1 Reports without targets
</commit_message>
<xml_diff>
--- a/sales_analysis_q1.xlsx
+++ b/sales_analysis_q1.xlsx
@@ -1194,13 +1194,13 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>145500000</v>
+        <v>48500000</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>159936565</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>1.099220378006873</v>
+        <v>3.297661134020619</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>0.25</v>
@@ -1218,13 +1218,13 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>21000000</v>
+        <v>7000000</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>15769084</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>0.7509087619047619</v>
+        <v>2.252726285714286</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>0.25</v>
@@ -1242,13 +1242,13 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>9000000</v>
+        <v>3000000</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>5635949</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>0.6262165555555556</v>
+        <v>1.878649666666667</v>
       </c>
       <c r="E15" s="10" t="n">
         <v>0.25</v>
@@ -1266,13 +1266,13 @@
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>4500000</v>
+        <v>1500000</v>
       </c>
       <c r="C16" s="9" t="n">
         <v>2102784</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>0.4672853333333333</v>
+        <v>1.401856</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>0.25</v>
@@ -1290,13 +1290,13 @@
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>180000000</v>
+        <v>60000000</v>
       </c>
       <c r="C17" s="9" t="n">
         <v>183444382</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>1.019135455555556</v>
+        <v>3.057406366666667</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>0.25</v>

</xml_diff>

<commit_message>
Customer sales report and market analysis updatesS
</commit_message>
<xml_diff>
--- a/sales_analysis_q1.xlsx
+++ b/sales_analysis_q1.xlsx
@@ -22,7 +22,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bonface_Kitheka" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dennis_Rudiga" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WALK_IN-BOMAS" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unknown" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -311,12 +310,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Rep Performance'!$B$4:$B$13</f>
+              <f>'Rep Performance'!$B$4:$B$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Rep Performance'!$D$4:$D$13</f>
+              <f>'Rep Performance'!$D$4:$D$12</f>
             </numRef>
           </val>
         </ser>
@@ -335,12 +334,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Rep Performance'!$B$4:$B$13</f>
+              <f>'Rep Performance'!$B$4:$B$12</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Rep Performance'!$E$4:$E$13</f>
+              <f>'Rep Performance'!$E$4:$E$12</f>
             </numRef>
           </val>
         </ser>
@@ -447,12 +446,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'GENERAL HARDWAR'!$A$6:$A$15</f>
+              <f>'GENERAL HARDWAR'!$A$6:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'GENERAL HARDWAR'!$B$6:$B$15</f>
+              <f>'GENERAL HARDWAR'!$B$6:$B$14</f>
             </numRef>
           </val>
         </ser>
@@ -505,12 +504,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'PAINTS'!$A$6:$A$15</f>
+              <f>'PAINTS'!$A$6:$A$14</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'PAINTS'!$B$6:$B$15</f>
+              <f>'PAINTS'!$B$6:$B$14</f>
             </numRef>
           </val>
         </ser>
@@ -648,7 +647,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>14</row>
+      <row>13</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7200000" cy="4320000"/>
@@ -675,7 +674,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="3600000"/>
@@ -702,7 +701,7 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>16</row>
+      <row>15</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="5760000" cy="3600000"/>
@@ -1105,7 +1104,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>183444382</v>
+        <v>183447102</v>
       </c>
     </row>
     <row r="6">
@@ -1115,7 +1114,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>16495300.6764</v>
+        <v>16495840.4128</v>
       </c>
     </row>
     <row r="7">
@@ -1125,7 +1124,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>0.08991990104335819</v>
+        <v>0.08992150997730125</v>
       </c>
     </row>
     <row r="8">
@@ -1135,7 +1134,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>2478978.135135135</v>
+        <v>2479014.891891892</v>
       </c>
     </row>
     <row r="9">
@@ -1145,7 +1144,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>222909.4686</v>
+        <v>222916.7623351351</v>
       </c>
     </row>
     <row r="11">
@@ -1197,10 +1196,10 @@
         <v>48500000</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>159936565</v>
+        <v>159937385</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>3.297661134020619</v>
+        <v>3.297678041237114</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>0.25</v>
@@ -1221,10 +1220,10 @@
         <v>7000000</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>15769084</v>
+        <v>15770984</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>2.252726285714286</v>
+        <v>2.252997714285714</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>0.25</v>
@@ -1293,10 +1292,10 @@
         <v>60000000</v>
       </c>
       <c r="C17" s="9" t="n">
-        <v>183444382</v>
+        <v>183447102</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>3.057406366666667</v>
+        <v>3.0574517</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>0.25</v>
@@ -1497,35 +1496,35 @@
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sales 27% below team average - needs improvement</t>
+          <t xml:space="preserve">  Sales 35% below team average - needs improvement</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Excellent margin at 15.1% (Team avg: 11.3%)</t>
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Paints Dept Head: 46.4% of dept sales, 17.5% margin</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Paints Dept Head: 46.4% of dept sales, 17.5% margin</t>
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Good paints leadership with 46.4% of dept sales</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Good paints leadership with 46.4% of dept sales</t>
+          <t xml:space="preserve">  Selling across all 4 categories - excellent product range</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Selling across all 4 categories - excellent product range</t>
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Best margin in ELECTRICALS: 35.5%</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1717,7 @@
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sales 28% below team average - needs improvement</t>
+          <t xml:space="preserve">  Sales 35% below team average - needs improvement</t>
         </is>
       </c>
     </row>
@@ -1939,14 +1938,14 @@
     <row r="14">
       <c r="A14" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sales 66% below team average - needs improvement</t>
+          <t xml:space="preserve">  Sales 69% below team average - needs improvement</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Excellent margin at 18.2% (Team avg: 11.3%)</t>
+          <t xml:space="preserve">  Excellent margin at 18.2% (Team avg: 12.5%)</t>
         </is>
       </c>
     </row>
@@ -2161,14 +2160,14 @@
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sales 71% below team average - needs improvement</t>
+          <t xml:space="preserve">  Sales 73% below team average - needs improvement</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Excellent margin at 16.3% (Team avg: 11.3%)</t>
+          <t xml:space="preserve">  Excellent margin at 16.3% (Team avg: 12.5%)</t>
         </is>
       </c>
     </row>
@@ -2382,14 +2381,14 @@
     <row r="13">
       <c r="A13" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sales 93% below team average - needs improvement</t>
+          <t xml:space="preserve">  Sales 94% below team average - needs improvement</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Excellent margin at 17.5% (Team avg: 11.3%)</t>
+          <t xml:space="preserve">  Excellent margin at 17.5% (Team avg: 12.5%)</t>
         </is>
       </c>
     </row>
@@ -2643,196 +2642,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="11" t="inlineStr">
-        <is>
-          <t>Unknown - General Hardware Team</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>Total Sales</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>Total Profit</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>Margin %</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>Items Sold</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="inlineStr">
-        <is>
-          <t>Sales Rank</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9" t="n">
-        <v>-2720</v>
-      </c>
-      <c r="B4" s="9" t="n">
-        <v>-539.7364</v>
-      </c>
-      <c r="C4" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="9" t="n">
-        <v>-5</v>
-      </c>
-      <c r="E4" s="8" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Sales (KES)</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
-        <is>
-          <t>Profit (KES)</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Margin %</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>GENERAL HARDWARE</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n">
-        <v>-820</v>
-      </c>
-      <c r="C7" s="9" t="n">
-        <v>-244.0176</v>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="9" t="n">
-        <v>-4</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>PAINTS</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>-1900</v>
-      </c>
-      <c r="C8" s="9" t="n">
-        <v>-295.7188</v>
-      </c>
-      <c r="D8" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="9" t="n">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>Performance Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Sales 100% below team average - needs improvement</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Margin at 0.0% below team average of 11.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  General Hardware: -0.0% of dept, 0.0% margin</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Limited to 2 categories - expand into PLUMBING, ELECTRICALS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Best margin in GENERAL HARDWARE: 0.0%</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2921,7 +2737,7 @@
         <v>85596.75</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>0.4041138201768424</v>
+        <v>0.4041078283155436</v>
       </c>
     </row>
     <row r="5">
@@ -2951,7 +2767,7 @@
         <v>55812</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>0.2120749110757723</v>
+        <v>0.2120717666065938</v>
       </c>
     </row>
     <row r="6">
@@ -2981,7 +2797,7 @@
         <v>43417.5</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>0.168201128121765</v>
+        <v>0.1681986341762979</v>
       </c>
     </row>
     <row r="7">
@@ -3011,7 +2827,7 @@
         <v>15973</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>0.0726702112905262</v>
+        <v>0.07266913379749111</v>
       </c>
     </row>
     <row r="8">
@@ -3041,7 +2857,7 @@
         <v>19440.15</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>0.07200524680009007</v>
+        <v>0.07200417916659158</v>
       </c>
     </row>
     <row r="9">
@@ -3071,7 +2887,7 @@
         <v>14234.75</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>0.03435450533448334</v>
+        <v>0.03435399595464855</v>
       </c>
     </row>
     <row r="10">
@@ -3101,7 +2917,7 @@
         <v>21242.5</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>0.02947197369064156</v>
+        <v>0.02947153670489709</v>
       </c>
     </row>
     <row r="11">
@@ -3131,7 +2947,7 @@
         <v>2331.75</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>0.006706092531086616</v>
+        <v>0.006705993098762607</v>
       </c>
     </row>
     <row r="12">
@@ -3161,37 +2977,7 @@
         <v>229</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>0.000416938361186771</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>General Hardware Team</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="n">
-        <v>-2720</v>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>-539.7364</v>
-      </c>
-      <c r="F13" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="9" t="n">
-        <v>-5</v>
-      </c>
-      <c r="H13" s="10" t="n">
-        <v>-1.482738239429976e-05</v>
+        <v>0.0004169321791739179</v>
       </c>
     </row>
   </sheetData>
@@ -3209,7 +2995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3237,7 +3023,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Total Sales: KES 159,936,565  |  Total Profit: KES 11,856,014</t>
+          <t>Total Sales: KES 159,937,385  |  Total Profit: KES 11,856,258</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3078,7 @@
         <v>83530.75</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>0.4553885473281236</v>
+        <v>0.4553862125481169</v>
       </c>
     </row>
     <row r="7">
@@ -3314,7 +3100,7 @@
         <v>48282</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.2267186743694289</v>
+        <v>0.2267175119813294</v>
       </c>
     </row>
     <row r="8">
@@ -3336,7 +3122,7 @@
         <v>35510.5</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.1644166985829663</v>
+        <v>0.1644158556174968</v>
       </c>
     </row>
     <row r="9">
@@ -3358,7 +3144,7 @@
         <v>17965.15</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.07556838550334002</v>
+        <v>0.07556799806374226</v>
       </c>
     </row>
     <row r="10">
@@ -3380,7 +3166,7 @@
         <v>8969.5</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.03541802338946069</v>
+        <v>0.03541784180102732</v>
       </c>
     </row>
     <row r="11">
@@ -3402,7 +3188,7 @@
         <v>5303.5</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.01903360873106159</v>
+        <v>0.0190335111456274</v>
       </c>
     </row>
     <row r="12">
@@ -3424,7 +3210,7 @@
         <v>4722.25</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0.0184206094460013</v>
+        <v>0.01842051500341837</v>
       </c>
     </row>
     <row r="13">
@@ -3446,7 +3232,7 @@
         <v>1319.75</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>0.004735314904380996</v>
+        <v>0.004735290626391071</v>
       </c>
     </row>
     <row r="14">
@@ -3468,29 +3254,7 @@
         <v>133</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.0003052647779449308</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>-820</v>
-      </c>
-      <c r="C15" s="9" t="n">
-        <v>-244.0176</v>
-      </c>
-      <c r="D15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>-4</v>
-      </c>
-      <c r="F15" s="10" t="n">
-        <v>-5.12703270824905e-06</v>
+        <v>0.000305263212850454</v>
       </c>
     </row>
   </sheetData>
@@ -3508,7 +3272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -3536,7 +3300,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Total Sales: KES 15,769,084  |  Total Profit: KES 2,725,590</t>
+          <t>Total Sales: KES 15,770,984  |  Total Profit: KES 2,725,886</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3355,7 @@
         <v>6013.5</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>0.4637891459009287</v>
+        <v>0.4637332711769918</v>
       </c>
     </row>
     <row r="7">
@@ -3613,7 +3377,7 @@
         <v>3329</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0.2351461885801357</v>
+        <v>0.2351178594816912</v>
       </c>
     </row>
     <row r="8">
@@ -3635,7 +3399,7 @@
         <v>1913</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.0976115670383898</v>
+        <v>0.09759980734239537</v>
       </c>
     </row>
     <row r="9">
@@ -3657,7 +3421,7 @@
         <v>969.5</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>0.05646776946587386</v>
+        <v>0.05646096654463666</v>
       </c>
     </row>
     <row r="10">
@@ -3679,7 +3443,7 @@
         <v>741</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>0.05563354218926096</v>
+        <v>0.05562683977106311</v>
       </c>
     </row>
     <row r="11">
@@ -3701,7 +3465,7 @@
         <v>760</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.04506285843870195</v>
+        <v>0.04505742951739727</v>
       </c>
     </row>
     <row r="12">
@@ -3723,7 +3487,7 @@
         <v>904</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>0.03352001929852108</v>
+        <v>0.033515980993957</v>
       </c>
     </row>
     <row r="13">
@@ -3745,7 +3509,7 @@
         <v>247</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>0.01208440515631726</v>
+        <v>0.01208294929473012</v>
       </c>
     </row>
     <row r="14">
@@ -3767,29 +3531,7 @@
         <v>5</v>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.0008049928581774313</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>-1900</v>
-      </c>
-      <c r="C15" s="9" t="n">
-        <v>-295.7188</v>
-      </c>
-      <c r="D15" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="9" t="n">
-        <v>-1</v>
-      </c>
-      <c r="F15" s="10" t="n">
-        <v>-0.0001204889263066897</v>
+        <v>0.0008048958771374062</v>
       </c>
     </row>
   </sheetData>
@@ -4543,14 +4285,14 @@
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Outstanding! Sales 304% above team average</t>
+          <t xml:space="preserve">  Outstanding! Sales 264% above team average</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Margin at 6.1% below team average of 11.3%</t>
+          <t xml:space="preserve">  Margin at 6.1% below team average of 12.5%</t>
         </is>
       </c>
     </row>
@@ -4765,14 +4507,14 @@
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Outstanding! Sales 112% above team average</t>
+          <t xml:space="preserve">  Outstanding! Sales 91% above team average</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Margin at 8.6% below team average of 11.3%</t>
+          <t xml:space="preserve">  Margin at 8.6% below team average of 12.5%</t>
         </is>
       </c>
     </row>
@@ -4811,7 +4553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4986,26 +4728,33 @@
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Outstanding! Sales 68% above team average</t>
+          <t xml:space="preserve">  Outstanding! Sales 51% above team average</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Margin at 9.4% below team average of 12.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  General Hardware: 16.4% of dept, 8.0% margin</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  Selling across all 4 categories - excellent product range</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  Best margin in PLUMBING: 31.9%</t>
         </is>

</xml_diff>